<commit_message>
feat(roadmap): Activity Timeline — unified feed over ideas, backlog, runs, research
Day 7 of the 100-Day Roadmap. Rather than wiring a generic audit-log emit
call into every service that creates something (broad, cross-cutting, and
risky to bolt onto code that already works), the timeline is derived from
the timestamped rows those services already write — the same read-only,
don't-touch-the-writers approach run_todo.py uses for per-run checklists.

Category filter (idea/feature/run/research) and cursor-based pagination
over (timestamp, id) for a stable, gap-free "load more". Each event deep
links to its source page — verified live, including a click-through from
a Run event straight to the matching row in Logs & Traces.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -4119,12 +4119,12 @@
       </c>
       <c r="N8" s="136" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="O8" s="147" t="inlineStr">
         <is>
-          <t>New: cross-feature activity feed.</t>
+          <t>Activity Timeline shipped as a derived feed over ideas/backlog/runs/research (not a generic audit-log wiring — see the code comment for why). Category filter + cursor pagination + deep links verified live.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(roadmap): Pins & Favorites across ideas, backlog, and documents
Day 8 of the 100-Day Roadmap. A generic Pin(entity_type, entity_id,
order_index) row rather than a `pinned` column on each of the three
tables — one ordering scheme instead of three kept in sync. This also
replaces the ad-hoc idea-only pin field added with the Idea Inbox.

Dangling pins clean themselves up when the list is next read, rather
than needing a sweep or a delete hook in every service that can delete
a pinnable thing. Reordering is keyboard-operable (arrow controls), not
drag-only, per the roadmap's accessibility DoD.

Pinned items get their own group at the top of the ⌘K palette, including
on an empty query — verified live end-to-end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -4218,12 +4218,12 @@
       </c>
       <c r="N9" s="136" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="O9" s="147" t="inlineStr">
         <is>
-          <t>New: pins/favorites.</t>
+          <t>Pins shipped as a generic Pin(entity_type, entity_id, order_index) across ideas/features/documents. Pinned strip on Dashboard, keyboard reorder (arrow buttons, not drag-only), dangling-pin cleanup on read, and command-palette boost — all verified live.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(roadmap): Today Home — one endpoint for today's actionable slice
Day 1 of the 100-Day Roadmap. GET /projects/{id}/home assembles pending
asks, untriaged ideas, in-flight sessions, failed runs, and top-Pareto
backlog in a single round-trip, so the landing screen doesn't make five.

Every section is capped — a home screen that grows with the database
stops being a home screen. Sections are ordered by what's blocked on the
builder; top backlog is the one forward-looking section and only renders
when nothing else is waiting, since the existing "Today's priority" card
already covers it with real Wizard/YOLO actions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -3530,12 +3530,12 @@
       </c>
       <c r="N2" s="136" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="O2" s="147" t="inlineStr">
         <is>
-          <t>Dashboard has a 'Today's priority' card; upgrading to a real daily agenda.</t>
+          <t>Today Home shipped: single GET /projects/{id}/home aggregating pending asks, untriaged ideas, in-flight sessions, failed runs, and top-Pareto backlog. Every section capped. Time-aware greeting and clean-slate state. Verified live.</t>
         </is>
       </c>
     </row>
@@ -6398,12 +6398,12 @@
       </c>
       <c r="N32" s="136" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="O32" s="147" t="inlineStr">
         <is>
-          <t>Backend (whisper.cpp) already shipped; only the frontend page is missing.</t>
+          <t>Transcribe page shipped this batch (whisper.cpp, fully offline) — model download, upload, segment transcript. Verified end-to-end with real synthesized audio.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(roadmap): first-run onboarding checklist with derived step state
Day 10 of the 100-Day Roadmap, completing Phase 1.

Each step's done-state is derived from real data — an Idea row exists, a
Node exists — rather than tracked in a parallel checklist table. A stored
checklist can drift from reality (mark a step done, then delete the thing
it was about); a derived one cannot. The only persisted state is whether
the builder dismissed the card.

Verified live against a project mid-way through the loop: capturing an
idea flipped the checklist from 2/4 to 3/4 with nothing written to it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -4416,12 +4416,12 @@
       </c>
       <c r="N11" s="136" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="O11" s="147" t="inlineStr">
         <is>
-          <t>New: first-run onboarding checklist.</t>
+          <t>Onboarding checklist shipped. Step completion is derived from real data (an Idea row exists, a Node exists) rather than a stored checklist, so it can never disagree with the app. Only the dismissed flag is persisted. Verified live: capturing an idea flipped 2/4 to 3/4.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(roadmap): Daily Streak & Momentum (D5) — closes Phase 1
Streak and 14-day sparkline on Today Home, derived from the Activity
Timeline feed rather than AuditEntry: the audit log only ever recorded
node create/update/verify, never idea captures, runs, or research, which
are exactly the qualifying actions a build streak should reward.

Day boundaries come from a client-supplied UTC offset — the browser is
the only component that reliably knows the user's timezone, and a streak
is a local-calendar concept (11:59pm and 12:01am are different days to a
person, the same day to UTC). 21 tests cover all six roadmap test cases
including the timezone boundary and the same-day dedupe.

Also adds parallel Lane assignments (A–H) to the roadmap tracker and
reconciles the stale Mind Map tab, which claimed 0/47 built when all
three phases had in fact shipped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -29,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="40">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -226,6 +226,27 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00166534"/>
+    </font>
   </fonts>
   <fills count="23">
     <fill>
@@ -410,7 +431,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="148">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -813,6 +834,15 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3344,7 +3374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3362,6 +3392,7 @@
     <col width="30" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="32" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3438,6 +3469,11 @@
       <c r="O1" s="141" t="inlineStr">
         <is>
           <t>Note</t>
+        </is>
+      </c>
+      <c r="P1" s="148" t="inlineStr">
+        <is>
+          <t>Lane</t>
         </is>
       </c>
     </row>
@@ -3538,6 +3574,11 @@
           <t>Today Home shipped: single GET /projects/{id}/home aggregating pending asks, untriaged ideas, in-flight sessions, failed runs, and top-Pareto backlog. Every section capped. Time-aware greeting and clean-slate state. Verified live.</t>
         </is>
       </c>
+      <c r="P2" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="222.1153846153846" customHeight="1">
       <c r="A3" s="35" t="n">
@@ -3637,6 +3678,11 @@
           <t>In-app quick-capture shipped (⌘I overlay, works from any page). OS-global hotkey still deferred — needs the Tauri capabilities work already deferred for reveal-in-Finder.</t>
         </is>
       </c>
+      <c r="P3" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="216.3461538461538" customHeight="1">
       <c r="A4" s="30" t="n">
@@ -3736,6 +3782,11 @@
           <t>Idea Inbox shipped: capture, list by status, triage into Backlog (Pareto-scored feature) or Research (creates a pending brief). Verified live end-to-end.</t>
         </is>
       </c>
+      <c r="P4" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="194.1346153846154" customHeight="1">
       <c r="A5" s="35" t="n">
@@ -3835,6 +3886,11 @@
           <t>Superseded — Command Palette (⌘K) already ships.</t>
         </is>
       </c>
+      <c r="P5" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="201.6346153846154" customHeight="1">
       <c r="A6" s="30" t="n">
@@ -3926,7 +3982,17 @@
       </c>
       <c r="N6" s="146" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Streak + 14-day sparkline on Today Home. Derived from the Activity Timeline feed (AuditEntry never recorded ideas/runs/research, so it was the wrong source). Day boundaries use a client-supplied UTC offset; 21 tests cover all 6 roadmap test cases.</t>
+        </is>
+      </c>
+      <c r="P6" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
         </is>
       </c>
     </row>
@@ -4028,6 +4094,11 @@
           <t>Superseded — Automations 'digest' action covers this.</t>
         </is>
       </c>
+      <c r="P7" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="187.5" customHeight="1">
       <c r="A8" s="30" t="n">
@@ -4127,6 +4198,11 @@
           <t>Activity Timeline shipped as a derived feed over ideas/backlog/runs/research (not a generic audit-log wiring — see the code comment for why). Category filter + cursor pagination + deep links verified live.</t>
         </is>
       </c>
+      <c r="P8" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="188.6538461538462" customHeight="1">
       <c r="A9" s="35" t="n">
@@ -4226,6 +4302,11 @@
           <t>Pins shipped as a generic Pin(entity_type, entity_id, order_index) across ideas/features/documents. Pinned strip on Dashboard, keyboard reorder (arrow buttons, not drag-only), dangling-pin cleanup on read, and command-palette boost — all verified live.</t>
         </is>
       </c>
+      <c r="P9" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="185.4807692307692" customHeight="1">
       <c r="A10" s="30" t="n">
@@ -4325,6 +4406,11 @@
           <t>Superseded — Global Search already ships.</t>
         </is>
       </c>
+      <c r="P10" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="214.3269230769231" customHeight="1">
       <c r="A11" s="35" t="n">
@@ -4424,6 +4510,11 @@
           <t>Onboarding checklist shipped. Step completion is derived from real data (an Idea row exists, a Node exists) rather than a stored checklist, so it can never disagree with the app. Only the dismissed flag is persisted. Verified live: capturing an idea flipped 2/4 to 3/4.</t>
         </is>
       </c>
+      <c r="P11" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="210.8653846153846" customHeight="1">
       <c r="A12" s="43" t="n">
@@ -4517,6 +4608,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P12" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="209.4230769230769" customHeight="1">
       <c r="A13" s="35" t="n">
@@ -4609,6 +4705,11 @@
       <c r="N13" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P13" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
         </is>
       </c>
     </row>
@@ -4707,6 +4808,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P14" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="194.4230769230769" customHeight="1">
       <c r="A15" s="35" t="n">
@@ -4801,6 +4907,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P15" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="210.8653846153846" customHeight="1">
       <c r="A16" s="43" t="n">
@@ -4895,6 +5006,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P16" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="202.2115384615385" customHeight="1">
       <c r="A17" s="35" t="n">
@@ -4989,6 +5105,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P17" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="175.0961538461538" customHeight="1">
       <c r="A18" s="43" t="n">
@@ -5080,6 +5201,11 @@
       <c r="N18" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P18" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
         </is>
       </c>
     </row>
@@ -5178,6 +5304,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P19" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="169.6153846153846" customHeight="1">
       <c r="A20" s="43" t="n">
@@ -5273,6 +5404,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P20" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="208.8461538461538" customHeight="1">
       <c r="A21" s="35" t="n">
@@ -5369,6 +5505,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P21" s="149" t="inlineStr">
+        <is>
+          <t>Lane B — Documents &amp; Editor</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="204.5192307692308" customHeight="1">
       <c r="A22" s="50" t="n">
@@ -5462,6 +5603,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P22" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="185.7692307692308" customHeight="1">
       <c r="A23" s="35" t="n">
@@ -5555,6 +5701,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P23" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="184.3269230769231" customHeight="1">
       <c r="A24" s="50" t="n">
@@ -5648,6 +5799,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P24" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="180.2884615384615" customHeight="1">
       <c r="A25" s="35" t="n">
@@ -5746,6 +5902,11 @@
           <t>Superseded — wigolo already does embeddings + reranking for search.</t>
         </is>
       </c>
+      <c r="P25" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="158.0769230769231" customHeight="1">
       <c r="A26" s="50" t="n">
@@ -5839,6 +6000,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P26" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="165.5769230769231" customHeight="1">
       <c r="A27" s="35" t="n">
@@ -5930,6 +6096,11 @@
       <c r="N27" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P27" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
         </is>
       </c>
     </row>
@@ -6026,6 +6197,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P28" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="172.5" customHeight="1">
       <c r="A29" s="35" t="n">
@@ -6120,6 +6296,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P29" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="180.2884615384615" customHeight="1">
       <c r="A30" s="50" t="n">
@@ -6211,6 +6392,11 @@
       <c r="N30" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P30" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
         </is>
       </c>
     </row>
@@ -6307,6 +6493,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P31" s="149" t="inlineStr">
+        <is>
+          <t>Lane C — AI Copilot &amp; Model Ops</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="216.6346153846154" customHeight="1">
       <c r="A32" s="56" t="n">
@@ -6406,6 +6597,11 @@
           <t>Transcribe page shipped this batch (whisper.cpp, fully offline) — model download, upload, segment transcript. Verified end-to-end with real synthesized audio.</t>
         </is>
       </c>
+      <c r="P32" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="176.8269230769231" customHeight="1">
       <c r="A33" s="35" t="n">
@@ -6498,6 +6694,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P33" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="165.5769230769231" customHeight="1">
       <c r="A34" s="56" t="n">
@@ -6591,6 +6792,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P34" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="167.5961538461538" customHeight="1">
       <c r="A35" s="35" t="n">
@@ -6684,6 +6890,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P35" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="160.3846153846154" customHeight="1">
       <c r="A36" s="56" t="n">
@@ -6777,6 +6988,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P36" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="162.1153846153846" customHeight="1">
       <c r="A37" s="35" t="n">
@@ -6870,6 +7086,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P37" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="169.3269230769231" customHeight="1">
       <c r="A38" s="56" t="n">
@@ -6963,6 +7184,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P38" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="152.8846153846154" customHeight="1">
       <c r="A39" s="35" t="n">
@@ -7056,6 +7282,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P39" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="167.5961538461538" customHeight="1">
       <c r="A40" s="56" t="n">
@@ -7149,6 +7380,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P40" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="162.4038461538462" customHeight="1">
       <c r="A41" s="35" t="n">
@@ -7240,6 +7476,11 @@
       <c r="N41" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P41" s="149" t="inlineStr">
+        <is>
+          <t>Lane A — Daily Home &amp; Capture</t>
         </is>
       </c>
     </row>
@@ -7337,6 +7578,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P42" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="163.8461538461538" customHeight="1">
       <c r="A43" s="35" t="n">
@@ -7431,6 +7677,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P43" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="169.0384615384615" customHeight="1">
       <c r="A44" s="62" t="n">
@@ -7525,6 +7776,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P44" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="160.3846153846154" customHeight="1">
       <c r="A45" s="35" t="n">
@@ -7619,6 +7875,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P45" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="162.9807692307692" customHeight="1">
       <c r="A46" s="62" t="n">
@@ -7713,6 +7974,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P46" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="169.9038461538462" customHeight="1">
       <c r="A47" s="35" t="n">
@@ -7807,6 +8073,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P47" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="161.8269230769231" customHeight="1">
       <c r="A48" s="62" t="n">
@@ -7901,6 +8172,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P48" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="159.5192307692308" customHeight="1">
       <c r="A49" s="35" t="n">
@@ -7995,6 +8271,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P49" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="155.1923076923077" customHeight="1">
       <c r="A50" s="62" t="n">
@@ -8089,6 +8370,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P50" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="167.0192307692308" customHeight="1">
       <c r="A51" s="35" t="n">
@@ -8183,6 +8469,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P51" s="149" t="inlineStr">
+        <is>
+          <t>Lane D — Planning &amp; PM</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="175.6730769230769" customHeight="1">
       <c r="A52" s="68" t="n">
@@ -8277,6 +8568,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P52" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="162.6923076923077" customHeight="1">
       <c r="A53" s="35" t="n">
@@ -8371,6 +8667,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P53" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="158.6538461538462" customHeight="1">
       <c r="A54" s="68" t="n">
@@ -8465,6 +8766,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P54" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="143.9423076923077" customHeight="1">
       <c r="A55" s="35" t="n">
@@ -8559,6 +8865,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P55" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="151.7307692307692" customHeight="1">
       <c r="A56" s="68" t="n">
@@ -8653,6 +8964,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P56" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="159.5192307692308" customHeight="1">
       <c r="A57" s="35" t="n">
@@ -8752,6 +9068,11 @@
           <t>Superseded — Slack/Telegram connectors + Automations digest already ship.</t>
         </is>
       </c>
+      <c r="P57" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="158.0769230769231" customHeight="1">
       <c r="A58" s="68" t="n">
@@ -8846,6 +9167,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P58" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="152.8846153846154" customHeight="1">
       <c r="A59" s="35" t="n">
@@ -8940,6 +9266,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P59" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="148.5576923076923" customHeight="1">
       <c r="A60" s="68" t="n">
@@ -9034,6 +9365,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P60" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="175.3846153846154" customHeight="1">
       <c r="A61" s="35" t="n">
@@ -9128,6 +9464,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P61" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="236.8269230769231" customHeight="1">
       <c r="A62" s="74" t="n">
@@ -9221,6 +9562,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P62" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="229.3269230769231" customHeight="1">
       <c r="A63" s="35" t="n">
@@ -9316,6 +9662,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P63" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="207.6923076923077" customHeight="1">
       <c r="A64" s="74" t="n">
@@ -9411,6 +9762,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P64" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="215.1923076923077" customHeight="1">
       <c r="A65" s="35" t="n">
@@ -9506,6 +9862,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P65" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="196.1538461538462" customHeight="1">
       <c r="A66" s="74" t="n">
@@ -9601,6 +9962,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P66" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="202.2115384615385" customHeight="1">
       <c r="A67" s="35" t="n">
@@ -9696,6 +10062,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P67" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="201.0576923076923" customHeight="1">
       <c r="A68" s="74" t="n">
@@ -9791,6 +10162,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P68" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="188.9423076923077" customHeight="1">
       <c r="A69" s="35" t="n">
@@ -9886,6 +10262,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P69" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="195.2884615384615" customHeight="1">
       <c r="A70" s="74" t="n">
@@ -9981,6 +10362,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P70" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="198.4615384615385" customHeight="1">
       <c r="A71" s="35" t="n">
@@ -10074,6 +10460,11 @@
       <c r="N71" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P71" s="149" t="inlineStr">
+        <is>
+          <t>Lane E — Integrations &amp; Server</t>
         </is>
       </c>
     </row>
@@ -10170,6 +10561,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P72" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="183.75" customHeight="1">
       <c r="A73" s="35" t="n">
@@ -10264,6 +10660,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P73" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="166.7307692307692" customHeight="1">
       <c r="A74" s="80" t="n">
@@ -10358,6 +10759,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P74" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="155.7692307692308" customHeight="1">
       <c r="A75" s="35" t="n">
@@ -10452,6 +10858,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P75" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="161.25" customHeight="1">
       <c r="A76" s="80" t="n">
@@ -10546,6 +10957,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P76" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="160.9615384615385" customHeight="1">
       <c r="A77" s="35" t="n">
@@ -10640,6 +11056,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P77" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="156.3461538461538" customHeight="1">
       <c r="A78" s="80" t="n">
@@ -10735,6 +11156,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P78" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="160.9615384615385" customHeight="1">
       <c r="A79" s="35" t="n">
@@ -10829,6 +11255,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P79" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="157.2115384615385" customHeight="1">
       <c r="A80" s="80" t="n">
@@ -10923,6 +11354,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P80" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="174.8076923076923" customHeight="1">
       <c r="A81" s="35" t="n">
@@ -11017,6 +11453,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P81" s="149" t="inlineStr">
+        <is>
+          <t>Lane F — Habit &amp; Delight</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="222.1153846153846" customHeight="1">
       <c r="A82" s="87" t="n">
@@ -11111,6 +11552,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P82" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="195" customHeight="1">
       <c r="A83" s="35" t="n">
@@ -11205,6 +11651,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P83" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="186.6346153846154" customHeight="1">
       <c r="A84" s="87" t="n">
@@ -11299,6 +11750,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P84" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="188.0769230769231" customHeight="1">
       <c r="A85" s="35" t="n">
@@ -11393,6 +11849,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P85" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="203.3653846153846" customHeight="1">
       <c r="A86" s="87" t="n">
@@ -11487,6 +11948,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P86" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="186.6346153846154" customHeight="1">
       <c r="A87" s="35" t="n">
@@ -11581,6 +12047,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P87" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="193.5576923076923" customHeight="1">
       <c r="A88" s="87" t="n">
@@ -11675,6 +12146,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P88" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="182.8846153846154" customHeight="1">
       <c r="A89" s="35" t="n">
@@ -11769,6 +12245,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P89" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="189.5192307692308" customHeight="1">
       <c r="A90" s="87" t="n">
@@ -11863,6 +12344,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P90" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="192.6923076923077" customHeight="1">
       <c r="A91" s="35" t="n">
@@ -11957,6 +12443,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P91" s="149" t="inlineStr">
+        <is>
+          <t>Lane G — Quality &amp; Trust</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="197.8846153846154" customHeight="1">
       <c r="A92" s="94" t="n">
@@ -12051,6 +12542,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P92" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="194.7115384615385" customHeight="1">
       <c r="A93" s="35" t="n">
@@ -12145,6 +12641,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P93" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="188.6538461538462" customHeight="1">
       <c r="A94" s="94" t="n">
@@ -12238,6 +12739,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P94" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="206.8269230769231" customHeight="1">
       <c r="A95" s="35" t="n">
@@ -12331,6 +12837,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P95" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="181.4423076923077" customHeight="1">
       <c r="A96" s="94" t="n">
@@ -12424,6 +12935,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P96" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="176.5384615384615" customHeight="1">
       <c r="A97" s="35" t="n">
@@ -12517,6 +13033,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P97" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="177.1153846153846" customHeight="1">
       <c r="A98" s="94" t="n">
@@ -12610,6 +13131,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P98" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="184.3269230769231" customHeight="1">
       <c r="A99" s="35" t="n">
@@ -12703,6 +13229,11 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="P99" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="188.3653846153846" customHeight="1">
       <c r="A100" s="94" t="n">
@@ -12794,6 +13325,11 @@
       <c r="N100" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P100" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
         </is>
       </c>
     </row>
@@ -12888,6 +13424,11 @@
       <c r="N101" s="146" t="inlineStr">
         <is>
           <t>Not started</t>
+        </is>
+      </c>
+      <c r="P101" s="149" t="inlineStr">
+        <is>
+          <t>Lane H — Scale &amp; Ecosystem</t>
         </is>
       </c>
     </row>
@@ -13000,7 +13541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13008,12 +13549,13 @@
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="115" t="inlineStr">
-        <is>
-          <t>Interactive Mind Mapping — planned feature (docs verified 2026-07-25; status 0/47 steps, nothing built yet)</t>
+      <c r="A1" s="150" t="inlineStr">
+        <is>
+          <t>Interactive Mind Mapping — SHIPPED (verified 2026-07-27). All 3 phases built: canvas CRUD, AI generate/expand/regroup/chat-edit, export JSON/Markdown/Mermaid/PNG/SVG + import with validation.</t>
         </is>
       </c>
     </row>
@@ -13133,6 +13675,11 @@
           <t>Roadmap placement</t>
         </is>
       </c>
+      <c r="F10" s="151" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="67.5" customHeight="1">
       <c r="A11" s="108" t="inlineStr">
@@ -13160,6 +13707,11 @@
           <t>Extends 100-Day Roadmap Phase 2 'Living Documents' (Days 11–20) — a visual editing surface alongside the text docs.</t>
         </is>
       </c>
+      <c r="F11" s="152" t="inlineStr">
+        <is>
+          <t>Done — React Flow canvas, node inspector, toolbar, shortcuts, persistence</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="62.7" customHeight="1">
       <c r="A12" s="108" t="inlineStr">
@@ -13187,6 +13739,11 @@
           <t>Pairs with Phase 3 'AI Copilot' (Days 21–30) — reuses the local LLM + next-best-action theme.</t>
         </is>
       </c>
+      <c r="F12" s="152" t="inlineStr">
+        <is>
+          <t>Done — generate_map / expand_node / regroup_map / chat_edit via local Ollama</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="66" customHeight="1">
       <c r="A13" s="108" t="inlineStr">
@@ -13212,6 +13769,11 @@
       <c r="E13" s="119" t="inlineStr">
         <is>
           <t>Feeds Phase 7 'Collaboration &amp; Sharing' (Days 61–70) export/publish and project-level exports.</t>
+        </is>
+      </c>
+      <c r="F13" s="152" t="inlineStr">
+        <is>
+          <t>Done — JSON/Markdown/Mermaid server-side; PNG/SVG client-side; import validated</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): reconcile OW parity tracker against Phase 6/7 work
Deliverables (row 43) is genuinely Done now — share links, real PDF, and
self-contained offline bundles are deliverable objects distinct from
documents, which was the gap. Refreshed the notes on the messaging and
connector rows so they describe what actually ships versus what still
needs third-party credentials.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -15270,7 +15270,7 @@
       </c>
       <c r="F33" s="127" t="inlineStr">
         <is>
-          <t>Mentions parsed and routed; signature-verified webhook. Needs a Slack app + bot token from your workspace to run.</t>
+          <t>Mentions parsed and routed; signature-verified webhook. @mentions of MEMBERS now also work in-app (D70). Slack itself still needs an app + bot token from your workspace to run end-to-end.</t>
         </is>
       </c>
     </row>
@@ -15462,7 +15462,7 @@
       </c>
       <c r="F39" s="127" t="inlineStr">
         <is>
-          <t>Two connectors of the 25+ OpenWorker ships. The interface is there; the rest is volume.</t>
+          <t>Two messaging connectors plus outbound webhooks (any endpoint, HMAC-signed) and a recipe engine, which together cover the generic integration case. The named 25+ SaaS connectors each need their own OAuth credentials.</t>
         </is>
       </c>
     </row>
@@ -15580,7 +15580,7 @@
       </c>
       <c r="D43" s="129" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E43" s="126" t="inlineStr">
@@ -15590,7 +15590,7 @@
       </c>
       <c r="F43" s="127" t="inlineStr">
         <is>
-          <t>Generated documents are browsable and exportable (md/json/mermaid/png/svg). No 'deliverable' object distinct from a document.</t>
+          <t>Deliverables now exist as objects distinct from documents: a read-only share link (revocable, expirable), a real 285-page PDF (ReportLab), and a self-contained offline HTML bundle (159 entries, zero external fetches) — alongside the existing md/json/mermaid/png/svg exports.</t>
         </is>
       </c>
     </row>
@@ -15846,7 +15846,7 @@
       </c>
       <c r="F51" s="127" t="inlineStr">
         <is>
-          <t>Deliberately deferred: an OAuth broker conflicts with local-first unless optional.</t>
+          <t>Deliberately deferred: an OAuth broker conflicts with local-first unless optional. Outbound webhooks + API keys give the same integration reach without a broker.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): pending-goals tab — 39 goals across 11 themes
Breaks the remaining work into sized, prioritised goals with explicit
blockers. The 150-minute block cap turns out to be a seam rather than a
bug: it exposes nine missing scheduling capabilities, three of them P0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -9,15 +9,16 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="100-Day Roadmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature · Mind Map" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Features" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Next Tasks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Connectors" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Tools" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Providers" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Configs" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · GUI Screens" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending · Goals" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature · Mind Map" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Features" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Next Tasks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Connectors" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Tools" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Providers" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · Configs" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OW · GUI Screens" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="44">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -247,6 +248,26 @@
       <name val="Arial"/>
       <color rgb="00166534"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00DC2626"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006B7280"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009CA3AF"/>
+    </font>
   </fonts>
   <fills count="23">
     <fill>
@@ -431,7 +452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -843,6 +864,24 @@
     </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1639,6 +1678,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="107" t="inlineStr">
+        <is>
+          <t>Model providers — provider-agnostic (aisuite + native OpenAI/Anthropic/Gemini). Bring your own key or run local via Ollama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="inlineStr">
+        <is>
+          <t>Native SDK</t>
+        </is>
+      </c>
+      <c r="C2" s="29" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="54" customHeight="1">
+      <c r="A3" s="111" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B3" s="112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" s="109" t="inlineStr">
+        <is>
+          <t>OpenAIProvider; default provider. env OPENAI_API_KEY; recommended gpt-5.6-sol. Optional custom base_url also serves Azure OpenAI /openai/v1, OpenRouter, vLLM, and any OpenAI-compliant gateway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="49.75" customHeight="1">
+      <c r="A4" s="113" t="inlineStr">
+        <is>
+          <t>Claude (Anthropic)</t>
+        </is>
+      </c>
+      <c r="B4" s="114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" s="110" t="inlineStr">
+        <is>
+          <t>AnthropicProvider — native Messages API. env ANTHROPIC_API_KEY; recommended claude-fable-5. Extended thinking on by default (hidden thinking_budget profile override; 0 = off).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28.75" customHeight="1">
+      <c r="A5" s="111" t="inlineStr">
+        <is>
+          <t>Gemini (Google)</t>
+        </is>
+      </c>
+      <c r="B5" s="112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" s="109" t="inlineStr">
+        <is>
+          <t>GeminiProvider — native Google GenAI API. env GEMINI_API_KEY; recommended gemini-3.6-flash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="43" customHeight="1">
+      <c r="A6" s="113" t="inlineStr">
+        <is>
+          <t>Ollama (local models)</t>
+        </is>
+      </c>
+      <c r="B6" s="114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C6" s="110" t="inlineStr">
+        <is>
+          <t>Local, keyless; reached via OpenAIProvider against the OpenAI-compatible /v1 endpoint (default http://localhost:11434). Recommended qwen3-coder:30b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45.25" customHeight="1">
+      <c r="A7" s="111" t="inlineStr">
+        <is>
+          <t>Z AI (GLM)</t>
+        </is>
+      </c>
+      <c r="B7" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C7" s="109" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API via OpenAIProvider. base https://api.z.ai/api/paas/v4; env ZAI_API_KEY; recommended glm-5.2. China mainland endpoint variant available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32.5" customHeight="1">
+      <c r="A8" s="113" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="B8" s="114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C8" s="110" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API. base https://api.deepseek.com; env DEEPSEEK_API_KEY; recommended deepseek-v4-flash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="41.75" customHeight="1">
+      <c r="A9" s="111" t="inlineStr">
+        <is>
+          <t>Kimi (Moonshot AI)</t>
+        </is>
+      </c>
+      <c r="B9" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C9" s="109" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API. base https://api.moonshot.ai/v1; env MOONSHOT_API_KEY; recommended kimi-k2.6. China mainland endpoint variant available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="31.25" customHeight="1">
+      <c r="A10" s="113" t="inlineStr">
+        <is>
+          <t>MiniMax</t>
+        </is>
+      </c>
+      <c r="B10" s="114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C10" s="110" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API. base https://api.minimax.io/v1; env MINIMAX_API_KEY; recommended MiniMax-M2.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="49.25" customHeight="1">
+      <c r="A11" s="111" t="inlineStr">
+        <is>
+          <t>Qwen (Alibaba)</t>
+        </is>
+      </c>
+      <c r="B11" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" s="109" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API. base https://dashscope-intl.aliyuncs.com/compatible-mode/v1; env DASHSCOPE_API_KEY; recommended qwen3-max. China (Beijing) endpoint variant available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="27.75" customHeight="1">
+      <c r="A12" s="113" t="inlineStr">
+        <is>
+          <t>xAI (Grok)</t>
+        </is>
+      </c>
+      <c r="B12" s="114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C12" s="110" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API. base https://api.x.ai/v1; env XAI_API_KEY; recommended grok-4.3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="33.25" customHeight="1">
+      <c r="A13" s="111" t="inlineStr">
+        <is>
+          <t>Mistral</t>
+        </is>
+      </c>
+      <c r="B13" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C13" s="109" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API. base https://api.mistral.ai/v1; env MISTRAL_API_KEY; recommended mistral-large-latest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40.25" customHeight="1">
+      <c r="A14" s="113" t="inlineStr">
+        <is>
+          <t>Meta (Muse Spark)</t>
+        </is>
+      </c>
+      <c r="B14" s="114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C14" s="110" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible API. base https://api.meta.ai/v1; env META_API_KEY; recommended muse-spark-1.1 (public preview, US-only as of 2026-07).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="47.75" customHeight="1">
+      <c r="A15" s="111" t="inlineStr">
+        <is>
+          <t>Together AI</t>
+        </is>
+      </c>
+      <c r="B15" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C15" s="109" t="inlineStr">
+        <is>
+          <t>Reseller via OpenAI-compatible API (many labs' models under Together's namespace). base https://api.together.xyz/v1; env TOGETHER_API_KEY; recommended zai-org/GLM-5.2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="43.25" customHeight="1">
+      <c r="A16" s="113" t="inlineStr">
+        <is>
+          <t>Fireworks AI</t>
+        </is>
+      </c>
+      <c r="B16" s="114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C16" s="110" t="inlineStr">
+        <is>
+          <t>Reseller via OpenAI-compatible API. base https://api.fireworks.ai/inference/v1; env FIREWORKS_API_KEY; recommended accounts/fireworks/models/glm-5p2.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2945,7 +3268,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13878,6 +14201,1642 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="74" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="132" t="inlineStr">
+        <is>
+          <t>Pending work as of 2026-07-27. Sized S (&lt;half day) / M (1-2 days) / L (3+ days). 'Blocked by' names what must exist first — external means credentials or infra I cannot supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="148" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="148" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="C2" s="148" t="inlineStr">
+        <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="D2" s="148" t="inlineStr">
+        <is>
+          <t>Why it matters</t>
+        </is>
+      </c>
+      <c r="E2" s="148" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="F2" s="148" t="inlineStr">
+        <is>
+          <t>Blocked by</t>
+        </is>
+      </c>
+      <c r="G2" s="148" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H2" s="148" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C3" s="153" t="inlineStr">
+        <is>
+          <t>Track time actually spent per work item</t>
+        </is>
+      </c>
+      <c r="D3" s="154" t="inlineStr">
+        <is>
+          <t>Nothing records that a 150-min block happened. Without it every later goal in this theme is guesswork.</t>
+        </is>
+      </c>
+      <c r="E3" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F3" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C4" s="153" t="inlineStr">
+        <is>
+          <t>Add remaining-effort so a capped block continues tomorrow</t>
+        </is>
+      </c>
+      <c r="D4" s="154" t="inlineStr">
+        <is>
+          <t>A 7-point item gets 150 min today, then the same 150 min tomorrow with no memory. Work never visibly shrinks.</t>
+        </is>
+      </c>
+      <c r="E4" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F4" s="153" t="inlineStr">
+        <is>
+          <t>Time tracking</t>
+        </is>
+      </c>
+      <c r="G4" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C5" s="153" t="inlineStr">
+        <is>
+          <t>Reconcile capacity units — planner counts points, scheduler counts minutes</t>
+        </is>
+      </c>
+      <c r="D5" s="154" t="inlineStr">
+        <is>
+          <t>capacity=8 admits one 7-point item, then the cap leaves 4h of the day empty. Measured 29.4% utilisation.</t>
+        </is>
+      </c>
+      <c r="E5" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F5" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C6" s="153" t="inlineStr">
+        <is>
+          <t>Suggest a work breakdown when an estimate exceeds one block</t>
+        </is>
+      </c>
+      <c r="D6" s="154" t="inlineStr">
+        <is>
+          <t>A 5.2h item should probably be three tasks. WBS already exists (D46); nothing offers it at the moment it is needed.</t>
+        </is>
+      </c>
+      <c r="E6" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F6" s="153" t="inlineStr">
+        <is>
+          <t>Remaining-effort</t>
+        </is>
+      </c>
+      <c r="G6" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C7" s="153" t="inlineStr">
+        <is>
+          <t>Project a completion date across days for oversized items</t>
+        </is>
+      </c>
+      <c r="D7" s="154" t="inlineStr">
+        <is>
+          <t>"This is 5.2h — it lands Thursday" is currently unanswerable.</t>
+        </is>
+      </c>
+      <c r="E7" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F7" s="153" t="inlineStr">
+        <is>
+          <t>Remaining-effort</t>
+        </is>
+      </c>
+      <c r="G7" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H7" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C8" s="153" t="inlineStr">
+        <is>
+          <t>Make max_block_minutes a user setting, not a constant</t>
+        </is>
+      </c>
+      <c r="D8" s="154" t="inlineStr">
+        <is>
+          <t>150 min is my guess about focus stamina, hard-coded. Some people work in 50s, some in 4h stretches.</t>
+        </is>
+      </c>
+      <c r="E8" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F8" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H8" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C9" s="153" t="inlineStr">
+        <is>
+          <t>Learn minutes-per-point from real cycle-time data</t>
+        </is>
+      </c>
+      <c r="D9" s="154" t="inlineStr">
+        <is>
+          <t>45 min/point is a guess. delivery_analytics already computes real cycle times — close the loop.</t>
+        </is>
+      </c>
+      <c r="E9" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F9" s="153" t="inlineStr">
+        <is>
+          <t>Time tracking</t>
+        </is>
+      </c>
+      <c r="G9" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H9" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C10" s="153" t="inlineStr">
+        <is>
+          <t>Reschedule the rest of the day when a block overruns</t>
+        </is>
+      </c>
+      <c r="D10" s="154" t="inlineStr">
+        <is>
+          <t>The buffer absorbs 15 min. A block that runs an hour long silently invalidates everything after it.</t>
+        </is>
+      </c>
+      <c r="E10" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F10" s="153" t="inlineStr">
+        <is>
+          <t>Time tracking</t>
+        </is>
+      </c>
+      <c r="G10" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H10" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="153" t="inlineStr">
+        <is>
+          <t>Time &amp; scheduling</t>
+        </is>
+      </c>
+      <c r="C11" s="153" t="inlineStr">
+        <is>
+          <t>Recurring commitments (standups, 1:1s) as fixed blocks</t>
+        </is>
+      </c>
+      <c r="D11" s="154" t="inlineStr">
+        <is>
+          <t>A schedule that ignores the meetings you already have is one you delete on day one.</t>
+        </is>
+      </c>
+      <c r="E11" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F11" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="153" t="inlineStr">
+        <is>
+          <t>Work Graph</t>
+        </is>
+      </c>
+      <c r="C12" s="153" t="inlineStr">
+        <is>
+          <t>UI reskin — serif display type, cream/dark palette, Daily Alignment layout</t>
+        </is>
+      </c>
+      <c r="D12" s="154" t="inlineStr">
+        <is>
+          <t>The last step of the agreed plan. The data model now supports every screen in the mockups.</t>
+        </is>
+      </c>
+      <c r="E12" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F12" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H12" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="153" t="inlineStr">
+        <is>
+          <t>Work Graph</t>
+        </is>
+      </c>
+      <c r="C13" s="153" t="inlineStr">
+        <is>
+          <t>Skill editor — currently you can fork and run, but not edit in the UI</t>
+        </is>
+      </c>
+      <c r="D13" s="154" t="inlineStr">
+        <is>
+          <t>The Skill Studio renders config beautifully and cannot change it. The API is complete; the form is not.</t>
+        </is>
+      </c>
+      <c r="E13" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F13" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H13" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="153" t="inlineStr">
+        <is>
+          <t>Work Graph</t>
+        </is>
+      </c>
+      <c r="C14" s="153" t="inlineStr">
+        <is>
+          <t>Attach skills to decisions and projects explicitly</t>
+        </is>
+      </c>
+      <c r="D14" s="154" t="inlineStr">
+        <is>
+          <t>Skill→project "unlocks" edges are inferred from blocked work. Real links would make the graph honest.</t>
+        </is>
+      </c>
+      <c r="E14" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F14" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H14" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="153" t="inlineStr">
+        <is>
+          <t>Work Graph</t>
+        </is>
+      </c>
+      <c r="C15" s="153" t="inlineStr">
+        <is>
+          <t>Decision templates (build-vs-buy, framework choice, hire-vs-contract)</t>
+        </is>
+      </c>
+      <c r="D15" s="154" t="inlineStr">
+        <is>
+          <t>Framing a good decision is a skill. Templates carry the framing so users do not have to.</t>
+        </is>
+      </c>
+      <c r="E15" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F15" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H15" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="153" t="inlineStr">
+        <is>
+          <t>Work Graph</t>
+        </is>
+      </c>
+      <c r="C16" s="153" t="inlineStr">
+        <is>
+          <t>Decision review — resurface decided forks to check the call held up</t>
+        </is>
+      </c>
+      <c r="D16" s="154" t="inlineStr">
+        <is>
+          <t>Deciding is append-only, which is the hard half. Learning from it needs the loop closed.</t>
+        </is>
+      </c>
+      <c r="E16" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F16" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H16" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="153" t="inlineStr">
+        <is>
+          <t>Work Graph</t>
+        </is>
+      </c>
+      <c r="C17" s="153" t="inlineStr">
+        <is>
+          <t>Graph filtering and focus mode for large projects</t>
+        </is>
+      </c>
+      <c r="D17" s="154" t="inlineStr">
+        <is>
+          <t>Currently caps at 12 project nodes and says what it hid. A real project needs filter-by-goal.</t>
+        </is>
+      </c>
+      <c r="E17" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F17" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H17" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="153" t="inlineStr">
+        <is>
+          <t>Roadmap · Partial</t>
+        </is>
+      </c>
+      <c r="C18" s="153" t="inlineStr">
+        <is>
+          <t>D29 — token-by-token streaming through providers.generate()</t>
+        </is>
+      </c>
+      <c r="D18" s="154" t="inlineStr">
+        <is>
+          <t>Per-call latency and run tracing ship. Real streaming needs a streaming transport in the provider layer.</t>
+        </is>
+      </c>
+      <c r="E18" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F18" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H18" s="156" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="153" t="inlineStr">
+        <is>
+          <t>Roadmap · Partial</t>
+        </is>
+      </c>
+      <c r="C19" s="153" t="inlineStr">
+        <is>
+          <t>D77 — keyboard cheat-sheet overlay and user rebinding</t>
+        </is>
+      </c>
+      <c r="D19" s="154" t="inlineStr">
+        <is>
+          <t>The shortcuts exist and are undiscoverable. A "?" overlay is most of the value.</t>
+        </is>
+      </c>
+      <c r="E19" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F19" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H19" s="156" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="153" t="inlineStr">
+        <is>
+          <t>Deferred · needs creds</t>
+        </is>
+      </c>
+      <c r="C20" s="153" t="inlineStr">
+        <is>
+          <t>One OAuth connector done properly end-to-end (GitHub first)</t>
+        </is>
+      </c>
+      <c r="D20" s="154" t="inlineStr">
+        <is>
+          <t>D51/D52. Building one against a live account teaches the shape for Jira, Linear, Notion.</t>
+        </is>
+      </c>
+      <c r="E20" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F20" s="153" t="inlineStr">
+        <is>
+          <t>External: GitHub OAuth app + test repo</t>
+        </is>
+      </c>
+      <c r="G20" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H20" s="156" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="153" t="inlineStr">
+        <is>
+          <t>Deferred · needs creds</t>
+        </is>
+      </c>
+      <c r="C21" s="153" t="inlineStr">
+        <is>
+          <t>Jira, Linear, Notion sync once the GitHub shape is proven</t>
+        </is>
+      </c>
+      <c r="D21" s="154" t="inlineStr">
+        <is>
+          <t>D53/D54/D55. Cheaper each time the first one is done, but each needs its own credentials.</t>
+        </is>
+      </c>
+      <c r="E21" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F21" s="153" t="inlineStr">
+        <is>
+          <t>External creds + GitHub connector</t>
+        </is>
+      </c>
+      <c r="G21" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H21" s="157" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="153" t="inlineStr">
+        <is>
+          <t>Deferred · needs creds</t>
+        </is>
+      </c>
+      <c r="C22" s="153" t="inlineStr">
+        <is>
+          <t>D57 Calendar time-blocking — write blocks to a real calendar</t>
+        </is>
+      </c>
+      <c r="D22" s="154" t="inlineStr">
+        <is>
+          <t>Pairs directly with the time-block scheduler. CalDAV would avoid a cloud dependency.</t>
+        </is>
+      </c>
+      <c r="E22" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F22" s="153" t="inlineStr">
+        <is>
+          <t>External: CalDAV or Google creds</t>
+        </is>
+      </c>
+      <c r="G22" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H22" s="156" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="153" t="inlineStr">
+        <is>
+          <t>Deferred · needs infra</t>
+        </is>
+      </c>
+      <c r="C23" s="153" t="inlineStr">
+        <is>
+          <t>D36 browser extension + D37 mobile PWA</t>
+        </is>
+      </c>
+      <c r="D23" s="154" t="inlineStr">
+        <is>
+          <t>The loopback capture endpoint already exists. Both need packaging and a hosted origin.</t>
+        </is>
+      </c>
+      <c r="E23" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F23" s="153" t="inlineStr">
+        <is>
+          <t>Store publishing / hosted origin</t>
+        </is>
+      </c>
+      <c r="G23" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H23" s="157" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="153" t="inlineStr">
+        <is>
+          <t>Deferred · needs design</t>
+        </is>
+      </c>
+      <c r="C24" s="153" t="inlineStr">
+        <is>
+          <t>D89 multi-device sync — conflict resolution model</t>
+        </is>
+      </c>
+      <c r="D24" s="154" t="inlineStr">
+        <is>
+          <t>A genuine design problem (CRDT vs last-writer-wins with a merge UI), not plumbing.</t>
+        </is>
+      </c>
+      <c r="E24" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F24" s="153" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="G24" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H24" s="157" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="153" t="inlineStr">
+        <is>
+          <t>Deferred · needs sandbox</t>
+        </is>
+      </c>
+      <c r="C25" s="153" t="inlineStr">
+        <is>
+          <t>D91 plugin SDK — sandbox and signing before executing third-party code</t>
+        </is>
+      </c>
+      <c r="D25" s="154" t="inlineStr">
+        <is>
+          <t>Dangerous in an app that also imports archives from other people. Needs a threat model first.</t>
+        </is>
+      </c>
+      <c r="E25" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F25" s="153" t="inlineStr">
+        <is>
+          <t>Security design</t>
+        </is>
+      </c>
+      <c r="G25" s="153" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H25" s="158" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="153" t="inlineStr">
+        <is>
+          <t>Deferred · needs hosting</t>
+        </is>
+      </c>
+      <c r="C26" s="153" t="inlineStr">
+        <is>
+          <t>D93 community marketplace</t>
+        </is>
+      </c>
+      <c r="D26" s="154" t="inlineStr">
+        <is>
+          <t>Needs hosting, moderation, and a trust story. Furthest from local-first.</t>
+        </is>
+      </c>
+      <c r="E26" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F26" s="153" t="inlineStr">
+        <is>
+          <t>Hosting + moderation</t>
+        </is>
+      </c>
+      <c r="G26" s="153" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H26" s="158" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="153" t="inlineStr">
+        <is>
+          <t>OW parity</t>
+        </is>
+      </c>
+      <c r="C27" s="153" t="inlineStr">
+        <is>
+          <t>Inline-vs-Inbox routing for approvals (OW row 16)</t>
+        </is>
+      </c>
+      <c r="D27" s="154" t="inlineStr">
+        <is>
+          <t>Everything goes to the Inbox. A fast yes/no for low-risk asks would cut the friction sharply.</t>
+        </is>
+      </c>
+      <c r="E27" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F27" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H27" s="156" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="153" t="inlineStr">
+        <is>
+          <t>OW parity</t>
+        </is>
+      </c>
+      <c r="C28" s="153" t="inlineStr">
+        <is>
+          <t>Per-task working folders and thread isolation (OW row 7)</t>
+        </is>
+      </c>
+      <c r="D28" s="154" t="inlineStr">
+        <is>
+          <t>Tasks run in-process today. Isolation matters once skills can be installed from elsewhere.</t>
+        </is>
+      </c>
+      <c r="E28" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F28" s="153" t="inlineStr">
+        <is>
+          <t>Plugin sandbox design</t>
+        </is>
+      </c>
+      <c r="G28" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H28" s="157" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="153" t="inlineStr">
+        <is>
+          <t>OW parity</t>
+        </is>
+      </c>
+      <c r="C29" s="153" t="inlineStr">
+        <is>
+          <t>Progressive skill disclosure for personas (OW row 32)</t>
+        </is>
+      </c>
+      <c r="D29" s="154" t="inlineStr">
+        <is>
+          <t>Personas contribute routing and prompts. The Skill object now gives this somewhere to land.</t>
+        </is>
+      </c>
+      <c r="E29" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F29" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H29" s="157" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="153" t="inlineStr">
+        <is>
+          <t>OW parity</t>
+        </is>
+      </c>
+      <c r="C30" s="153" t="inlineStr">
+        <is>
+          <t>OS-level reveal-in-Finder + OS-global capture hotkey (OW row 44, D2)</t>
+        </is>
+      </c>
+      <c r="D30" s="154" t="inlineStr">
+        <is>
+          <t>Both blocked on the same Tauri capabilities work. Worth doing together.</t>
+        </is>
+      </c>
+      <c r="E30" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F30" s="153" t="inlineStr">
+        <is>
+          <t>Tauri capabilities config</t>
+        </is>
+      </c>
+      <c r="G30" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H30" s="156" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="153" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C31" s="153" t="inlineStr">
+        <is>
+          <t>Fix suite-wide test isolation — every module shares one database</t>
+        </is>
+      </c>
+      <c r="D31" s="154" t="inlineStr">
+        <is>
+          <t>Modules set DOBBY_DB_PATH but src.main imports once. Three tests already broke on ordering.</t>
+        </is>
+      </c>
+      <c r="E31" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F31" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H31" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="153" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C32" s="153" t="inlineStr">
+        <is>
+          <t>D88 vault: extend encryption beyond settings to connector credentials</t>
+        </is>
+      </c>
+      <c r="D32" s="154" t="inlineStr">
+        <is>
+          <t>The vault protects six settings fields. Messaging and MCP credentials are still plaintext.</t>
+        </is>
+      </c>
+      <c r="E32" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F32" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H32" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="153" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C33" s="153" t="inlineStr">
+        <is>
+          <t>Frontend test coverage — there is currently none</t>
+        </is>
+      </c>
+      <c r="D33" s="154" t="inlineStr">
+        <is>
+          <t>1,334 backend tests and zero for the UI. Every bug I found in the UI was found by eye.</t>
+        </is>
+      </c>
+      <c r="E33" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F33" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H33" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="153" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C34" s="153" t="inlineStr">
+        <is>
+          <t>Deduplicate the three Markdown renderers</t>
+        </is>
+      </c>
+      <c r="D34" s="154" t="inlineStr">
+        <is>
+          <t>markdown.ts (preview), publish_service (bundles), and the PDF builder each parse Markdown separately.</t>
+        </is>
+      </c>
+      <c r="E34" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F34" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H34" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="153" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C35" s="153" t="inlineStr">
+        <is>
+          <t>Retire the seeded demo data or make it obviously fake</t>
+        </is>
+      </c>
+      <c r="D35" s="154" t="inlineStr">
+        <is>
+          <t>"Data Encryption", "Offline Syncing" look like real backlog items and pollute every screenshot.</t>
+        </is>
+      </c>
+      <c r="E35" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F35" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="153" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H35" s="156" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="153" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C36" s="153" t="inlineStr">
+        <is>
+          <t>Performance pass — the work graph and timeline read every row</t>
+        </is>
+      </c>
+      <c r="D36" s="154" t="inlineStr">
+        <is>
+          <t>Fine at 157 nodes. A project with 5,000 documents will not be.</t>
+        </is>
+      </c>
+      <c r="E36" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F36" s="153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H36" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="153" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="C37" s="153" t="inlineStr">
+        <is>
+          <t>Signed, notarised macOS build with auto-update</t>
+        </is>
+      </c>
+      <c r="D37" s="154" t="inlineStr">
+        <is>
+          <t>The open-core plan sells the signed build. Nothing is packaged yet.</t>
+        </is>
+      </c>
+      <c r="E37" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F37" s="153" t="inlineStr">
+        <is>
+          <t>Apple developer cert</t>
+        </is>
+      </c>
+      <c r="G37" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H37" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="153" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="C38" s="153" t="inlineStr">
+        <is>
+          <t>Wire licence verification into the packaged app</t>
+        </is>
+      </c>
+      <c r="D38" s="154" t="inlineStr">
+        <is>
+          <t>The Ed25519 licensing + clock-rollback detection is built and unused by any real build.</t>
+        </is>
+      </c>
+      <c r="E38" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F38" s="153" t="inlineStr">
+        <is>
+          <t>Signed build</t>
+        </is>
+      </c>
+      <c r="G38" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H38" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="153" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="C39" s="153" t="inlineStr">
+        <is>
+          <t>Billing — Lemon Squeezy / Paddle, after 1000 beta users</t>
+        </is>
+      </c>
+      <c r="D39" s="154" t="inlineStr">
+        <is>
+          <t>Your call: deferred until the product is complete. The licence layer is ready for it.</t>
+        </is>
+      </c>
+      <c r="E39" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F39" s="153" t="inlineStr">
+        <is>
+          <t>Signed build + beta</t>
+        </is>
+      </c>
+      <c r="G39" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H39" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="153" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="C40" s="153" t="inlineStr">
+        <is>
+          <t>Onboarding for a genuinely empty install</t>
+        </is>
+      </c>
+      <c r="D40" s="154" t="inlineStr">
+        <is>
+          <t>Every screen has been verified against a seeded project. A first-run user sees empty states we have barely tested.</t>
+        </is>
+      </c>
+      <c r="E40" s="154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F40" s="153" t="inlineStr">
+        <is>
+          <t>Demo-data retirement</t>
+        </is>
+      </c>
+      <c r="G40" s="153" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H40" s="155" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="153" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="C41" s="153" t="inlineStr">
+        <is>
+          <t>Windows and Linux builds</t>
+        </is>
+      </c>
+      <c r="D41" s="154" t="inlineStr">
+        <is>
+          <t>Tauri supports them; nothing has been built or tested outside macOS. OCR/keychain paths are macOS-specific.</t>
+        </is>
+      </c>
+      <c r="E41" s="154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F41" s="153" t="inlineStr">
+        <is>
+          <t>Signed build</t>
+        </is>
+      </c>
+      <c r="G41" s="153" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H41" s="157" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -13970,7 +15929,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14226,7 +16185,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16140,7 +18099,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16571,7 +18530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18137,7 +20096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19415,288 +21374,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="107" t="inlineStr">
-        <is>
-          <t>Model providers — provider-agnostic (aisuite + native OpenAI/Anthropic/Gemini). Bring your own key or run local via Ollama.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="29" t="inlineStr">
-        <is>
-          <t>Provider</t>
-        </is>
-      </c>
-      <c r="B2" s="29" t="inlineStr">
-        <is>
-          <t>Native SDK</t>
-        </is>
-      </c>
-      <c r="C2" s="29" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="54" customHeight="1">
-      <c r="A3" s="111" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="B3" s="112" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C3" s="109" t="inlineStr">
-        <is>
-          <t>OpenAIProvider; default provider. env OPENAI_API_KEY; recommended gpt-5.6-sol. Optional custom base_url also serves Azure OpenAI /openai/v1, OpenRouter, vLLM, and any OpenAI-compliant gateway.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="49.75" customHeight="1">
-      <c r="A4" s="113" t="inlineStr">
-        <is>
-          <t>Claude (Anthropic)</t>
-        </is>
-      </c>
-      <c r="B4" s="114" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C4" s="110" t="inlineStr">
-        <is>
-          <t>AnthropicProvider — native Messages API. env ANTHROPIC_API_KEY; recommended claude-fable-5. Extended thinking on by default (hidden thinking_budget profile override; 0 = off).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28.75" customHeight="1">
-      <c r="A5" s="111" t="inlineStr">
-        <is>
-          <t>Gemini (Google)</t>
-        </is>
-      </c>
-      <c r="B5" s="112" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C5" s="109" t="inlineStr">
-        <is>
-          <t>GeminiProvider — native Google GenAI API. env GEMINI_API_KEY; recommended gemini-3.6-flash.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="43" customHeight="1">
-      <c r="A6" s="113" t="inlineStr">
-        <is>
-          <t>Ollama (local models)</t>
-        </is>
-      </c>
-      <c r="B6" s="114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C6" s="110" t="inlineStr">
-        <is>
-          <t>Local, keyless; reached via OpenAIProvider against the OpenAI-compatible /v1 endpoint (default http://localhost:11434). Recommended qwen3-coder:30b.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45.25" customHeight="1">
-      <c r="A7" s="111" t="inlineStr">
-        <is>
-          <t>Z AI (GLM)</t>
-        </is>
-      </c>
-      <c r="B7" s="112" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C7" s="109" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API via OpenAIProvider. base https://api.z.ai/api/paas/v4; env ZAI_API_KEY; recommended glm-5.2. China mainland endpoint variant available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32.5" customHeight="1">
-      <c r="A8" s="113" t="inlineStr">
-        <is>
-          <t>DeepSeek</t>
-        </is>
-      </c>
-      <c r="B8" s="114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C8" s="110" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API. base https://api.deepseek.com; env DEEPSEEK_API_KEY; recommended deepseek-v4-flash.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.75" customHeight="1">
-      <c r="A9" s="111" t="inlineStr">
-        <is>
-          <t>Kimi (Moonshot AI)</t>
-        </is>
-      </c>
-      <c r="B9" s="112" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C9" s="109" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API. base https://api.moonshot.ai/v1; env MOONSHOT_API_KEY; recommended kimi-k2.6. China mainland endpoint variant available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="31.25" customHeight="1">
-      <c r="A10" s="113" t="inlineStr">
-        <is>
-          <t>MiniMax</t>
-        </is>
-      </c>
-      <c r="B10" s="114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C10" s="110" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API. base https://api.minimax.io/v1; env MINIMAX_API_KEY; recommended MiniMax-M2.5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="49.25" customHeight="1">
-      <c r="A11" s="111" t="inlineStr">
-        <is>
-          <t>Qwen (Alibaba)</t>
-        </is>
-      </c>
-      <c r="B11" s="112" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C11" s="109" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API. base https://dashscope-intl.aliyuncs.com/compatible-mode/v1; env DASHSCOPE_API_KEY; recommended qwen3-max. China (Beijing) endpoint variant available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="27.75" customHeight="1">
-      <c r="A12" s="113" t="inlineStr">
-        <is>
-          <t>xAI (Grok)</t>
-        </is>
-      </c>
-      <c r="B12" s="114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C12" s="110" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API. base https://api.x.ai/v1; env XAI_API_KEY; recommended grok-4.3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="33.25" customHeight="1">
-      <c r="A13" s="111" t="inlineStr">
-        <is>
-          <t>Mistral</t>
-        </is>
-      </c>
-      <c r="B13" s="112" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C13" s="109" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API. base https://api.mistral.ai/v1; env MISTRAL_API_KEY; recommended mistral-large-latest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40.25" customHeight="1">
-      <c r="A14" s="113" t="inlineStr">
-        <is>
-          <t>Meta (Muse Spark)</t>
-        </is>
-      </c>
-      <c r="B14" s="114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C14" s="110" t="inlineStr">
-        <is>
-          <t>OpenAI-compatible API. base https://api.meta.ai/v1; env META_API_KEY; recommended muse-spark-1.1 (public preview, US-only as of 2026-07).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="47.75" customHeight="1">
-      <c r="A15" s="111" t="inlineStr">
-        <is>
-          <t>Together AI</t>
-        </is>
-      </c>
-      <c r="B15" s="112" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C15" s="109" t="inlineStr">
-        <is>
-          <t>Reseller via OpenAI-compatible API (many labs' models under Together's namespace). base https://api.together.xyz/v1; env TOGETHER_API_KEY; recommended zai-org/GLM-5.2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="43.25" customHeight="1">
-      <c r="A16" s="113" t="inlineStr">
-        <is>
-          <t>Fireworks AI</t>
-        </is>
-      </c>
-      <c r="B16" s="114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C16" s="110" t="inlineStr">
-        <is>
-          <t>Reseller via OpenAI-compatible API. base https://api.fireworks.ai/inference/v1; env FIREWORKS_API_KEY; recommended accounts/fireworks/models/glm-5p2.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(roadmap): mark the three time-tracking P0s done
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -14299,7 +14299,7 @@
       </c>
       <c r="H3" s="155" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14339,7 +14339,7 @@
       </c>
       <c r="H4" s="155" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14379,7 @@
       </c>
       <c r="H5" s="155" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>